<commit_message>
Remove reviewer-attribution columns from manual-check outputs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/revision1/outputs/03_confidence_band_audit.xlsx
+++ b/revision1/outputs/03_confidence_band_audit.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="191">
   <si>
     <t>band</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Checked_By</t>
-  </si>
-  <si>
     <t>medium (0.5-0.9)</t>
   </si>
   <si>
@@ -590,9 +587,6 @@
   </si>
   <si>
     <t>Explicit two-phase mixed-method design</t>
-  </si>
-  <si>
-    <t>Claude (first pass) - authors to verify</t>
   </si>
 </sst>
 </file>
@@ -950,10 +944,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -984,1408 +978,1285 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2">
         <v>2018</v>
       </c>
       <c r="E2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F2">
         <v>0.594</v>
       </c>
       <c r="G2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J2" t="s">
-        <v>152</v>
-      </c>
-      <c r="K2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D3">
         <v>2012</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F3">
         <v>0.8663</v>
       </c>
       <c r="G3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J3" t="s">
-        <v>153</v>
-      </c>
-      <c r="K3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D4">
         <v>2022</v>
       </c>
       <c r="E4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F4">
         <v>0.8417</v>
       </c>
       <c r="G4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H4" t="s">
         <v>134</v>
       </c>
-      <c r="H4" t="s">
-        <v>135</v>
-      </c>
       <c r="I4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J4" t="s">
-        <v>154</v>
-      </c>
-      <c r="K4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D5">
         <v>2023</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F5">
         <v>0.6806</v>
       </c>
       <c r="G5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J5" t="s">
-        <v>155</v>
-      </c>
-      <c r="K5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6">
         <v>2013</v>
       </c>
       <c r="E6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F6">
         <v>0.7529</v>
       </c>
       <c r="G6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J6" t="s">
-        <v>156</v>
-      </c>
-      <c r="K6" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D7">
         <v>2018</v>
       </c>
       <c r="E7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F7">
         <v>0.8078</v>
       </c>
       <c r="G7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J7" t="s">
-        <v>157</v>
-      </c>
-      <c r="K7" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D8">
         <v>2000</v>
       </c>
       <c r="E8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F8">
         <v>0.6888</v>
       </c>
       <c r="G8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J8" t="s">
-        <v>158</v>
-      </c>
-      <c r="K8" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9">
         <v>2018</v>
       </c>
       <c r="E9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F9">
         <v>0.6894</v>
       </c>
       <c r="G9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J9" t="s">
-        <v>159</v>
-      </c>
-      <c r="K9" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D10">
         <v>2022</v>
       </c>
       <c r="E10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10">
         <v>0.7088</v>
       </c>
       <c r="G10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J10" t="s">
-        <v>160</v>
-      </c>
-      <c r="K10" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11">
         <v>2015</v>
       </c>
       <c r="E11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F11">
         <v>0.6743</v>
       </c>
       <c r="G11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J11" t="s">
-        <v>161</v>
-      </c>
-      <c r="K11" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D12">
         <v>2001</v>
       </c>
       <c r="E12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F12">
         <v>0.5325</v>
       </c>
       <c r="G12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J12" t="s">
-        <v>162</v>
-      </c>
-      <c r="K12" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D13">
         <v>2014</v>
       </c>
       <c r="E13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F13">
         <v>0.6191</v>
       </c>
       <c r="G13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J13" t="s">
-        <v>163</v>
-      </c>
-      <c r="K13" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D14">
         <v>2005</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F14">
         <v>0.7989000000000001</v>
       </c>
       <c r="G14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J14" t="s">
-        <v>164</v>
-      </c>
-      <c r="K14" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D15">
         <v>2005</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F15">
         <v>0.5925</v>
       </c>
       <c r="G15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J15" t="s">
-        <v>165</v>
-      </c>
-      <c r="K15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D16">
         <v>2021</v>
       </c>
       <c r="E16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F16">
         <v>0.7497</v>
       </c>
       <c r="G16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J16" t="s">
-        <v>166</v>
-      </c>
-      <c r="K16" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D17">
         <v>2009</v>
       </c>
       <c r="E17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F17">
         <v>0.6639</v>
       </c>
       <c r="G17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J17" t="s">
-        <v>167</v>
-      </c>
-      <c r="K17" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D18">
         <v>2006</v>
       </c>
       <c r="E18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F18">
         <v>0.8475</v>
       </c>
       <c r="G18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I18" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J18" t="s">
-        <v>168</v>
-      </c>
-      <c r="K18" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D19">
         <v>2002</v>
       </c>
       <c r="E19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F19">
         <v>0.7707000000000001</v>
       </c>
       <c r="G19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I19" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J19" t="s">
-        <v>169</v>
-      </c>
-      <c r="K19" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D20">
         <v>2009</v>
       </c>
       <c r="E20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F20">
         <v>0.597</v>
       </c>
       <c r="G20" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H20" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J20" t="s">
-        <v>170</v>
-      </c>
-      <c r="K20" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D21">
         <v>2009</v>
       </c>
       <c r="E21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F21">
         <v>0.6692</v>
       </c>
       <c r="G21" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
-      </c>
-      <c r="K21" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D22">
         <v>2013</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F22">
         <v>0.9805</v>
       </c>
       <c r="G22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J22" t="s">
-        <v>172</v>
-      </c>
-      <c r="K22" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D23">
         <v>2024</v>
       </c>
       <c r="E23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F23">
         <v>0.9986</v>
       </c>
       <c r="G23" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H23" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I23" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J23" t="s">
-        <v>173</v>
-      </c>
-      <c r="K23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D24">
         <v>2003</v>
       </c>
       <c r="E24" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F24">
         <v>0.9925</v>
       </c>
       <c r="G24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I24" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J24" t="s">
-        <v>174</v>
-      </c>
-      <c r="K24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D25">
         <v>2014</v>
       </c>
       <c r="E25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F25">
         <v>0.9999</v>
       </c>
       <c r="G25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J25" t="s">
-        <v>175</v>
-      </c>
-      <c r="K25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D26">
         <v>2021</v>
       </c>
       <c r="E26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F26">
         <v>0.9079</v>
       </c>
       <c r="G26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J26" t="s">
-        <v>176</v>
-      </c>
-      <c r="K26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D27">
         <v>2022</v>
       </c>
       <c r="E27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F27">
         <v>0.9722</v>
       </c>
       <c r="G27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I27" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J27" t="s">
-        <v>177</v>
-      </c>
-      <c r="K27" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D28">
         <v>2007</v>
       </c>
       <c r="E28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F28">
         <v>0.9853</v>
       </c>
       <c r="G28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J28" t="s">
-        <v>178</v>
-      </c>
-      <c r="K28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D29">
         <v>1997</v>
       </c>
       <c r="E29" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F29">
         <v>0.9227</v>
       </c>
       <c r="G29" t="s">
+        <v>138</v>
+      </c>
+      <c r="H29" t="s">
         <v>139</v>
       </c>
-      <c r="H29" t="s">
-        <v>140</v>
-      </c>
       <c r="I29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J29" t="s">
-        <v>179</v>
-      </c>
-      <c r="K29" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D30">
         <v>2021</v>
       </c>
       <c r="E30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J30" t="s">
-        <v>180</v>
-      </c>
-      <c r="K30" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D31">
         <v>2016</v>
       </c>
       <c r="E31" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F31">
         <v>0.9074</v>
       </c>
       <c r="G31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I31" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J31" t="s">
-        <v>181</v>
-      </c>
-      <c r="K31" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D32">
         <v>2021</v>
       </c>
       <c r="E32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F32">
         <v>0.9999</v>
       </c>
       <c r="G32" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H32" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I32" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J32" t="s">
-        <v>182</v>
-      </c>
-      <c r="K32" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D33">
         <v>2007</v>
       </c>
       <c r="E33" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F33">
         <v>0.9575</v>
       </c>
       <c r="G33" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H33" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J33" t="s">
-        <v>183</v>
-      </c>
-      <c r="K33" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D34">
         <v>2009</v>
       </c>
       <c r="E34" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F34">
         <v>0.9965000000000001</v>
       </c>
       <c r="G34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I34" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J34" t="s">
-        <v>184</v>
-      </c>
-      <c r="K34" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D35">
         <v>2008</v>
       </c>
       <c r="E35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F35">
         <v>0.9876</v>
       </c>
       <c r="G35" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H35" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J35" t="s">
-        <v>185</v>
-      </c>
-      <c r="K35" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D36">
         <v>2022</v>
       </c>
       <c r="E36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F36">
         <v>0.9653</v>
       </c>
       <c r="G36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I36" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J36" t="s">
-        <v>186</v>
-      </c>
-      <c r="K36" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37">
         <v>2023</v>
       </c>
       <c r="E37" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F37">
         <v>0.9688</v>
       </c>
       <c r="G37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J37" t="s">
-        <v>187</v>
-      </c>
-      <c r="K37" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D38">
         <v>2023</v>
       </c>
       <c r="E38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F38">
         <v>0.9579</v>
       </c>
       <c r="G38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J38" t="s">
-        <v>188</v>
-      </c>
-      <c r="K38" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D39">
         <v>1993</v>
       </c>
       <c r="E39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F39">
         <v>0.9998</v>
       </c>
       <c r="G39" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H39" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I39" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J39" t="s">
-        <v>189</v>
-      </c>
-      <c r="K39" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D40">
         <v>2014</v>
       </c>
       <c r="E40" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F40">
         <v>0.9989</v>
       </c>
       <c r="G40" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H40" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I40" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J40" t="s">
-        <v>190</v>
-      </c>
-      <c r="K40" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D41">
         <v>2018</v>
       </c>
       <c r="E41" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F41">
         <v>0.9201</v>
       </c>
       <c r="G41" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I41" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J41" t="s">
-        <v>191</v>
-      </c>
-      <c r="K41" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>